<commit_message>
Documenta a estrutura atual do app (ESTRUTURA.md): fluxo, o que abre por escopo x metodo, regras globais e pontos em aberto
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C42C902-4E46-4A99-B5AE-602C68254B95}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB67453F-A24C-4E84-B479-BE7660AFF1F4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
-    <sheet name="Planilha2" sheetId="2" r:id="rId2"/>
-    <sheet name="Planilha3" sheetId="3" r:id="rId3"/>
+    <sheet name="Planilha2" sheetId="2" r:id="rId1"/>
+    <sheet name="Planilha3" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,25 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
-  <si>
-    <t>ruido interno</t>
-  </si>
-  <si>
-    <t>ruido externo</t>
-  </si>
-  <si>
-    <t>ruido ferroviario</t>
-  </si>
-  <si>
-    <t>ruido aeronautico</t>
-  </si>
-  <si>
-    <t>ruido interno 10152</t>
-  </si>
-  <si>
-    <t>solicitei campo de fachada</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t>Ruído Ambiental – NBR 10151</t>
   </si>
@@ -199,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -221,12 +202,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -561,47 +536,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63AF6A2D-0495-4BB5-A527-58125004C2DD}">
-  <dimension ref="D5:E9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="5" spans="4:5" x14ac:dyDescent="0.3">
-      <c r="D5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="4:5" x14ac:dyDescent="0.3">
-      <c r="D6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="4:5" x14ac:dyDescent="0.3">
-      <c r="D7" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="4:5" x14ac:dyDescent="0.3">
-      <c r="D8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="4:5" x14ac:dyDescent="0.3">
-      <c r="D9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9526D981-1FA4-46DC-815A-C9E12F5EFA92}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -613,97 +547,97 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>21</v>
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>22</v>
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>22</v>
+        <v>2</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>22</v>
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="C5" s="9" t="s">
-        <v>22</v>
+      <c r="C5" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>22</v>
+        <v>9</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>22</v>
+        <v>11</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="6"/>
       <c r="B9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>22</v>
+        <v>12</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -722,7 +656,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74AA8FCB-3663-445A-9945-CAE71C4AAE1F}">
   <dimension ref="E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -732,7 +666,7 @@
   <sheetData>
     <row r="5" spans="5:5" ht="409.6" x14ac:dyDescent="0.3">
       <c r="E5" s="7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ruido/interno: divide subtipo em 10151 e 10152 (aba Padrao da planilha)
A aba "Padrao" de escopo_metodo_os.xlsx define que o Ambiente Interno deve
ser dividido por norma. Antes os dois usavam o MESMO formulario "interno".

- mapa-escopo: subtipoPorEscopo devolve interno10151 (NBR 10151 "Ambiente
  interno") ou interno10152 (NBR 10152).
- campo-ruido: dois cards de subtipo, FOTOS_POR_SUBTIPO/TIPOS_CARIMBO por
  subtipo (RUIDOINTERNO10151/RUIDOINTERNO10152) e helper ehInterno() nos 4
  pontos do formulario.
- Por ora os dois formularios sao IDENTICOS, exceto a nota: 10151 = "monitorar,
  preferencialmente, com pessoas"; 10152 = "sem pessoas". Resto a detalhar.
- service-worker: cache ecamp-v0.7.1. ESTRUTURA.md atualizado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB67453F-A24C-4E84-B479-BE7660AFF1F4}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F5D6088-A014-442F-9337-717A8FE22EE3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha2" sheetId="2" r:id="rId1"/>
+    <sheet name="Padrão" sheetId="2" r:id="rId1"/>
     <sheet name="Planilha3" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
   <si>
     <t>Ruído Ambiental – NBR 10151</t>
   </si>
@@ -116,6 +116,106 @@
 •	Ar Interno (MQAI)
 6.	Já selecionar em “Tipo de Monitoramento”: Outro quando os escopos forem
 •	Outros</t>
+  </si>
+  <si>
+    <t>Subtipo do monitoramento</t>
+  </si>
+  <si>
+    <t>Ambiente Externo</t>
+  </si>
+  <si>
+    <t>Ambiente Interno 10151</t>
+  </si>
+  <si>
+    <t>Ambiente Interno 10152</t>
+  </si>
+  <si>
+    <t>Aeronáutico</t>
+  </si>
+  <si>
+    <t>Ferroviário</t>
+  </si>
+  <si>
+    <t>ROMANEIO</t>
+  </si>
+  <si>
+    <t>**Checklist de Saída para Monitoramento de Ruído**
+**1. Antes de sair do laboratório**
+* Ordem de Serviço (OS) avaliada
+* Pontos amostrais identificados
+* Trajeto planejado
+* Acesso ao local confirmado com o cliente
+* EPIs disponíveis e em boas condições
+**2. Equipamentos e insumos**
+**Equipamentos**
+* Sonômetro com calibração válida
+* Calibrador acústico com calibração válida
+* Microfone com calibração válida
+* Termohigroanemômetro com calibração válida
+**Acessórios**
+* Tripé
+* Protetor de vento (windscreen)
+* Trena
+* Maleta/mochila
+**Alimentação e energia**
+* Carregador dos equipamentos
+* Baterias reservas
+* Power bank carregado
+* Celular carregado
+* Carregador do celular
+**3. Itens opcionais para monitoramentos de longa duração**
+* Cabo de extensão
+* Estação meteorológica com calibração válida
+**4. Itens opcionais para monitoramento online**
+* Roteador 4G
+* Internet móvel funcionando
+**5. Verificação final**
+* Equipamentos conferidos
+* Baterias carregadas
+* Materiais acondicionados para transporte
+* Equipe alinhada quanto ao serviço
+* Horário de saída confirmado</t>
+  </si>
+  <si>
+    <t>**🌍 Romaneio para Ensaios de Vibração**
+**1. Antes de sair do laboratório**
+* Ordem de Serviço (OS) avaliada
+* Pontos amostrais identificados
+* Trajeto planejado (chegada com antecedência mínima de 1 hora)
+* Acesso ao local confirmado com o cliente
+* EPIs disponíveis
+**2. Equipamentos e insumos**
+**Equipamentos**
+* Sismógrafo com calibração válida
+* Geofone com calibração válida
+* Microfone com calibração válida
+* Termohigroanemômetro com calibração válida
+**Acessórios**
+* Cabo de conexão entre sismógrafo e geofone
+* Tripé para o microfone
+* Protetor de vento (windscreen)
+* Trena métrica
+* Maleta de transporte
+* Notebook com software SISTEX (confirmar necessidade com o coordenador)
+**Alimentação e energia**
+* Carregador dos equipamentos
+* Baterias reservas
+* Power bank carregado
+* Celular carregado
+* Carregador do celular
+**3. Insumos para fixação do geofone**
+* Cravos para fixação no solo
+* Gesso de secagem rápida
+* Recipiente para preparo do gesso
+* Água para preparo do gesso
+* Fita adesiva (proteção dos furos do geofone)
+* Espátula para remoção do gesso
+**4. Verificação final**
+* Equipamentos conferidos
+* Baterias carregadas
+* Materiais acondicionados para transporte
+* Equipe alinhada quanto ao serviço
+* Horário de saída confirmado</t>
   </si>
 </sst>
 </file>
@@ -180,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -189,19 +289,26 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,15 +644,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9526D981-1FA4-46DC-815A-C9E12F5EFA92}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultRowHeight="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.77734375" customWidth="1"/>
+    <col min="1" max="1" width="34.21875" customWidth="1"/>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -555,102 +664,170 @@
       <c r="C1" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="D1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4" t="s">
+    <row r="3" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
+    <row r="4" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="D4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="D5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="4" t="s">
+      <c r="D6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="6"/>
-      <c r="B9" s="4" t="s">
+      <c r="D8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
-    </row>
+      <c r="D10" s="1"/>
+      <c r="E10" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-  </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -665,7 +842,7 @@
   </cols>
   <sheetData>
     <row r="5" spans="5:5" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="4" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruido/interno 10151 (tela por ponto): campo "Condicoes do ambiente"
Na tela de servico por ponto do Ambiente Interno 10151, antes do bloco
"Condicoes ambientais (somente no primeiro ponto)", novo titulo "Condicoes do
ambiente" com escolha obrigatoria: Ambiente vazio / Ambiente mobiliado.

- So no subtipo interno10151 e so no 1o ponto (a sala e unica por servico,
  como o bloco de clima ao lado). Radios (toque unico, bom p/ campo).
- Obrigatorio no 1o ponto: trava o salvamento se nao escolhido (interno10152
  nao exige). Valor em ponto.condAmbiente.
- service-worker: cache ecamp-v0.7.2. ESTRUTURA.md atualizado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F5D6088-A014-442F-9337-717A8FE22EE3}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{977BD2E8-9811-487F-B20E-7DB05721C60E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="39">
   <si>
     <t>Ruído Ambiental – NBR 10151</t>
   </si>
@@ -82,9 +82,6 @@
   </si>
   <si>
     <t>ok</t>
-  </si>
-  <si>
-    <t>Substituir "monitorar, preferencialmente, sem pessoas" para "monitorar, preferencialmente, com pessoas"</t>
   </si>
   <si>
     <t>Tipo de Monitoramento</t>
@@ -139,83 +136,49 @@
     <t>ROMANEIO</t>
   </si>
   <si>
-    <t>**Checklist de Saída para Monitoramento de Ruído**
-**1. Antes de sair do laboratório**
-* Ordem de Serviço (OS) avaliada
-* Pontos amostrais identificados
-* Trajeto planejado
-* Acesso ao local confirmado com o cliente
-* EPIs disponíveis e em boas condições
-**2. Equipamentos e insumos**
-**Equipamentos**
-* Sonômetro com calibração válida
-* Calibrador acústico com calibração válida
-* Microfone com calibração válida
-* Termohigroanemômetro com calibração válida
-**Acessórios**
-* Tripé
-* Protetor de vento (windscreen)
-* Trena
-* Maleta/mochila
-**Alimentação e energia**
-* Carregador dos equipamentos
-* Baterias reservas
-* Power bank carregado
-* Celular carregado
-* Carregador do celular
-**3. Itens opcionais para monitoramentos de longa duração**
-* Cabo de extensão
-* Estação meteorológica com calibração válida
-**4. Itens opcionais para monitoramento online**
-* Roteador 4G
-* Internet móvel funcionando
-**5. Verificação final**
-* Equipamentos conferidos
-* Baterias carregadas
-* Materiais acondicionados para transporte
-* Equipe alinhada quanto ao serviço
-* Horário de saída confirmado</t>
-  </si>
-  <si>
-    <t>**🌍 Romaneio para Ensaios de Vibração**
-**1. Antes de sair do laboratório**
-* Ordem de Serviço (OS) avaliada
-* Pontos amostrais identificados
-* Trajeto planejado (chegada com antecedência mínima de 1 hora)
-* Acesso ao local confirmado com o cliente
-* EPIs disponíveis
-**2. Equipamentos e insumos**
-**Equipamentos**
-* Sismógrafo com calibração válida
-* Geofone com calibração válida
-* Microfone com calibração válida
-* Termohigroanemômetro com calibração válida
-**Acessórios**
-* Cabo de conexão entre sismógrafo e geofone
-* Tripé para o microfone
-* Protetor de vento (windscreen)
-* Trena métrica
-* Maleta de transporte
-* Notebook com software SISTEX (confirmar necessidade com o coordenador)
-**Alimentação e energia**
-* Carregador dos equipamentos
-* Baterias reservas
-* Power bank carregado
-* Celular carregado
-* Carregador do celular
-**3. Insumos para fixação do geofone**
-* Cravos para fixação no solo
-* Gesso de secagem rápida
-* Recipiente para preparo do gesso
-* Água para preparo do gesso
-* Fita adesiva (proteção dos furos do geofone)
-* Espátula para remoção do gesso
-**4. Verificação final**
-* Equipamentos conferidos
-* Baterias carregadas
-* Materiais acondicionados para transporte
-* Equipe alinhada quanto ao serviço
-* Horário de saída confirmado</t>
+    <t>Sismografia – NBR 9653</t>
+  </si>
+  <si>
+    <t>Usual</t>
+  </si>
+  <si>
+    <t>Online</t>
+  </si>
+  <si>
+    <t>Patrimônio Espeleológico – CECAV</t>
+  </si>
+  <si>
+    <t>Áreas Habitadas – CETESB DD 215/2007</t>
+  </si>
+  <si>
+    <t>Vibração</t>
+  </si>
+  <si>
+    <t>TELA SERVIÇO (POR PONTO)</t>
+  </si>
+  <si>
+    <t>Ok</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Ler documento "ecamp_especificação_docx" item 8.2 (Vibração)</t>
+  </si>
+  <si>
+    <t>Ler documento "ecamp_especificação_docx" item 7.2 (Vibração)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ler documento "ecamp_especificação_docx" item 7.1 </t>
+  </si>
+  <si>
+    <t>OBSERVAÇÕES:</t>
+  </si>
+  <si>
+    <t>Mantenha sempre as alterações e versões que ajustei nas conversas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento de referência: </t>
   </si>
 </sst>
 </file>
@@ -253,7 +216,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -276,15 +239,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -294,8 +291,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -304,11 +301,26 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -644,189 +656,375 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9526D981-1FA4-46DC-815A-C9E12F5EFA92}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.21875" customWidth="1"/>
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.88671875" customWidth="1"/>
     <col min="4" max="4" width="22.33203125" customWidth="1"/>
-    <col min="5" max="5" width="46" customWidth="1"/>
+    <col min="5" max="6" width="46" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D2" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="16"/>
+      <c r="G2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="E3" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="16"/>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="16"/>
+    </row>
+    <row r="5" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="16"/>
+    </row>
+    <row r="6" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="E6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="16"/>
+    </row>
+    <row r="7" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="16"/>
+    </row>
+    <row r="8" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="16"/>
+    </row>
+    <row r="9" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="C9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="16"/>
+    </row>
+    <row r="10" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="10" t="s">
+      <c r="C10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="C11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+    </row>
+    <row r="17" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="15"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+    </row>
+    <row r="18" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="15"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+    </row>
+    <row r="19" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="15"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+    </row>
+    <row r="20" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="15"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+    </row>
+    <row r="21" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="15"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+    </row>
+    <row r="22" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+    </row>
+    <row r="23" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -842,8 +1040,8 @@
   </cols>
   <sheetData>
     <row r="5" spans="5:5" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="E5" s="4" t="s">
-        <v>17</v>
+      <c r="E5" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ruido/interno: montagem com resposta por norma (10151 fast / 10152 slow)
Na montagem do equipamento (tela de preparacao, apos calcular pontos), o check
de configuracao agora muda por subtipo:
- interno10151: "...(ponderacao A, fast (F), tempo de medicao, audio)"
- interno10152: "...(ponderacao A, slow (S), tempo de medicao, audio)"

CHECKS_MONTAGEM_INTERNO virou checksMontagemInterno(sub). Demais 4 itens
iguais; comprimento 5 mantido (validacao inalterada). Cache ecamp-v0.7.3.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{977BD2E8-9811-487F-B20E-7DB05721C60E}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DE705CC-6453-4ADD-A7A6-9C4CA447EDC0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="39">
   <si>
     <t>Ruído Ambiental – NBR 10151</t>
   </si>
@@ -79,9 +79,6 @@
   </si>
   <si>
     <t>Pátios / Manobras / Cruzamentos</t>
-  </si>
-  <si>
-    <t>ok</t>
   </si>
   <si>
     <t>Tipo de Monitoramento</t>
@@ -157,9 +154,6 @@
     <t>TELA SERVIÇO (POR PONTO)</t>
   </si>
   <si>
-    <t>Ok</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -179,6 +173,12 @@
   </si>
   <si>
     <t xml:space="preserve">Documento de referência: </t>
+  </si>
+  <si>
+    <t>e-CAMP</t>
+  </si>
+  <si>
+    <t>pronto. Não mexer.</t>
   </si>
 </sst>
 </file>
@@ -202,7 +202,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -212,6 +212,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -280,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -321,6 +327,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -664,6 +673,7 @@
     <col min="3" max="3" width="19.88671875" customWidth="1"/>
     <col min="4" max="4" width="22.33203125" customWidth="1"/>
     <col min="5" max="6" width="46" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
@@ -674,58 +684,61 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="17" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F2" s="16"/>
-      <c r="G2" t="s">
-        <v>31</v>
+      <c r="G2" s="10" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="17" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F3" s="16"/>
-      <c r="G3" t="s">
-        <v>13</v>
+      <c r="G3" s="10" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -736,15 +749,18 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F4" s="16"/>
+      <c r="G4" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -752,15 +768,18 @@
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F5" s="16"/>
+      <c r="G5" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
@@ -770,15 +789,18 @@
         <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F6" s="16"/>
+      <c r="G6" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
@@ -788,15 +810,18 @@
         <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F7" s="16"/>
+      <c r="G7" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -806,15 +831,18 @@
         <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F8" s="16"/>
+      <c r="G8" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
@@ -824,135 +852,144 @@
         <v>12</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F9" s="16"/>
+      <c r="G9" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="10" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="C10" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="F10" s="4" t="s">
-        <v>33</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G10" s="10"/>
     </row>
     <row r="11" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D11" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="F11" s="4" t="s">
-        <v>33</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G11" s="10"/>
     </row>
     <row r="12" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D12" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="F12" s="4" t="s">
-        <v>33</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G12" s="10"/>
     </row>
     <row r="13" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D13" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="F13" s="4" t="s">
-        <v>33</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G13" s="10"/>
     </row>
     <row r="14" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="D14" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="F14" s="4" t="s">
-        <v>33</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G14" s="10"/>
     </row>
     <row r="15" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="D15" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="F15" s="4" t="s">
-        <v>33</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G15" s="10"/>
     </row>
     <row r="16" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="15"/>
@@ -961,68 +998,75 @@
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
-    </row>
-    <row r="17" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="15"/>
       <c r="B17" s="11"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
-    </row>
-    <row r="18" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G17" s="10"/>
+    </row>
+    <row r="18" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
-    </row>
-    <row r="19" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G18" s="10"/>
+    </row>
+    <row r="19" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="15"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
-    </row>
-    <row r="20" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G19" s="10"/>
+    </row>
+    <row r="20" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="15"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
-    </row>
-    <row r="21" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G20" s="10"/>
+    </row>
+    <row r="21" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="15"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
-    </row>
-    <row r="22" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G21" s="10"/>
+    </row>
+    <row r="22" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
-    </row>
-    <row r="23" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G22" s="10"/>
+    </row>
+    <row r="23" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" t="s">
         <v>36</v>
-      </c>
-      <c r="C23" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1041,7 +1085,7 @@
   <sheetData>
     <row r="5" spans="5:5" ht="409.6" x14ac:dyDescent="0.3">
       <c r="E5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PWA: aviso "nova versao disponivel" com botao Atualizar (sem reload surpresa)
Resolve o "um refresh atrasado": antes a nova versao so aparecia no 2o abrir.
Agora o SW novo fica EM ESPERA e o app mostra um aviso; ao tocar em Atualizar
ele assume e a pagina recarrega. Nada recarrega sozinho (seguro em campo).

- service-worker: remove skipWaiting do install (fica em espera); escuta
  mensagem SKIP_WAITING para assumir sob comando. Cache ecamp-v0.7.4.
- app.js: detecta versao em espera (registro.waiting / updatefound) e mostra o
  aviso; controllerchange recarrega 1x, so quando ja havia controlador (nao na
  1a instalacao). Funcao mostrarAvisoAtualizacao.
- index.html + estilos.css: banner #aviso-atualizacao com botao #btn-atualizar.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DE705CC-6453-4ADD-A7A6-9C4CA447EDC0}"/>
+  <xr:revisionPtr revIDLastSave="117" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7852CFC-639C-4E02-89EB-3CB5C2252DE1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
@@ -672,7 +672,8 @@
     <col min="2" max="2" width="46" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.88671875" customWidth="1"/>
     <col min="4" max="4" width="22.33203125" customWidth="1"/>
-    <col min="5" max="6" width="46" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
+    <col min="6" max="6" width="51.88671875" customWidth="1"/>
     <col min="7" max="7" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -785,7 +786,7 @@
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="17" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -806,7 +807,7 @@
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -1091,4 +1092,237 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010012D067C7C505F94DA745333F0C70E18C" ma:contentTypeVersion="12" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="9a7942e81b10ac3f7052d292e3c7485f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ceff588c-4f4f-49af-b7d7-c9c79415ad32" xmlns:ns3="0ea24c86-fc74-4fa0-a83b-660477924ea4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3596c5fc9896945baf8297a4f7e536bd" ns2:_="" ns3:_="">
+    <xsd:import namespace="ceff588c-4f4f-49af-b7d7-c9c79415ad32"/>
+    <xsd:import namespace="0ea24c86-fc74-4fa0-a83b-660477924ea4"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ceff588c-4f4f-49af-b7d7-c9c79415ad32" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="12" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e9d251d0-a9ed-4942-8f9c-4135f39fc0f0" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="17" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="0ea24c86-fc74-4fa0-a83b-660477924ea4" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="13" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{2bd60ddc-46c7-4f89-952c-d01989346355}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="0ea24c86-fc74-4fa0-a83b-660477924ea4">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ceff588c-4f4f-49af-b7d7-c9c79415ad32">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0ea24c86-fc74-4fa0-a83b-660477924ea4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCA0AE08-2331-4162-B9EC-E40252058BA9}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5B55AC-A0C1-45C3-9411-3D2F7156D1B8}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB7D7E8-8145-4A74-B49E-03C8140943AB}"/>
 </file>
</xml_diff>

<commit_message>
Ruido/ferroviario "Patios/Manobras/Cruzamentos": instalacao, operacoes e ponto
Mudancas SO no metodo Patios / Manobras / Cruzamentos (Passagem intacta):

- Requisitos de instalacao proprios (4 itens: altura >=4 m, 2 m de superficies
  refletoras, protetor de vento, microfone direcionado p/ trafego). Obrigatorio.
- Checks do ponto: "curto periodo"/"longa duracao" em negrito; condicao
  ambiental separada em dois checks (chuva / vento) -> 5 checks no ponto.
- Abaixo da qtde de pontos: checklist "Operacoes em patios / manobras /
  cruzamentos" com sub-titulos em negrito (Manobras / Composicao parada /
  Cruzamentos-Ultrapassagens). NAO bloqueia o salvamento (orientacao de campo).

Implementacao: FERRO_PATIOS, CHECKS_INSTALACAO_FERRO_PATIOS,
CHECKS_PONTO_FERRO_PATIOS, OPERACOES_FERRO_PATIOS, checksPontoFerro(),
htmlOperacoesFerroPatios(); validacao por metodo. CSS .subgrupo-titulo.
Cache ecamp-v0.7.5.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7852CFC-639C-4E02-89EB-3CB5C2252DE1}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A839BED7-ADD2-4BFE-A667-046CD60D8FA6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
@@ -286,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -306,13 +306,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -329,6 +325,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -687,7 +686,7 @@
       <c r="C1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -704,20 +703,20 @@
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="11" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="16"/>
-      <c r="G2" s="10" t="s">
+      <c r="F2" s="14"/>
+      <c r="G2" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -725,20 +724,20 @@
       <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="15" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="11" t="s">
         <v>17</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="16"/>
-      <c r="G3" s="10" t="s">
+      <c r="F3" s="14"/>
+      <c r="G3" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -752,14 +751,14 @@
       <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="11" t="s">
         <v>17</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="16"/>
-      <c r="G4" s="10" t="s">
+      <c r="F4" s="14"/>
+      <c r="G4" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -767,18 +766,18 @@
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2"/>
+      <c r="B5" s="15"/>
       <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="16"/>
-      <c r="G5" s="10" t="s">
+      <c r="F5" s="14"/>
+      <c r="G5" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -786,20 +785,20 @@
       <c r="A6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="11" t="s">
         <v>20</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="16"/>
-      <c r="G6" s="10" t="s">
+      <c r="F6" s="14"/>
+      <c r="G6" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -807,20 +806,20 @@
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="11" t="s">
         <v>20</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="10" t="s">
+      <c r="F7" s="14"/>
+      <c r="G7" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -828,20 +827,20 @@
       <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="15" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="11" t="s">
         <v>21</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="16"/>
-      <c r="G8" s="10" t="s">
+      <c r="F8" s="14"/>
+      <c r="G8" s="7" t="s">
         <v>38</v>
       </c>
     </row>
@@ -849,25 +848,25 @@
       <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="16" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="12" t="s">
         <v>21</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="16"/>
-      <c r="G9" s="10" t="s">
+      <c r="F9" s="14"/>
+      <c r="G9" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -876,7 +875,7 @@
       <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="11" t="s">
         <v>30</v>
       </c>
       <c r="E10" s="4" t="s">
@@ -885,19 +884,19 @@
       <c r="F10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="10"/>
+      <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E11" s="4" t="s">
@@ -906,10 +905,10 @@
       <c r="F11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="10"/>
+      <c r="G11" s="7"/>
     </row>
     <row r="12" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="7" t="s">
         <v>26</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -918,7 +917,7 @@
       <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="4" t="s">
@@ -927,19 +926,19 @@
       <c r="F12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="10"/>
+      <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E13" s="4" t="s">
@@ -948,10 +947,10 @@
       <c r="F13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -960,7 +959,7 @@
       <c r="C14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E14" s="4" t="s">
@@ -969,19 +968,19 @@
       <c r="F14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="10"/>
+      <c r="G14" s="7"/>
     </row>
     <row r="15" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E15" s="4" t="s">
@@ -990,69 +989,69 @@
       <c r="F15" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="10"/>
+      <c r="G15" s="7"/>
     </row>
     <row r="16" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="15"/>
+      <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
     </row>
     <row r="17" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="15"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
     </row>
     <row r="18" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="15"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
     </row>
     <row r="19" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="15"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
     </row>
     <row r="20" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="15"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
     </row>
     <row r="21" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="15"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
     </row>
     <row r="22" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
     </row>
     <row r="23" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
@@ -1084,7 +1083,7 @@
     <col min="5" max="5" width="71.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="5:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="5:5" ht="388.8" x14ac:dyDescent="0.3">
       <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
@@ -1296,15 +1295,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ceff588c-4f4f-49af-b7d7-c9c79415ad32">
@@ -1315,14 +1305,49 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCA0AE08-2331-4162-B9EC-E40252058BA9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCA0AE08-2331-4162-B9EC-E40252058BA9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ceff588c-4f4f-49af-b7d7-c9c79415ad32"/>
+    <ds:schemaRef ds:uri="0ea24c86-fc74-4fa0-a83b-660477924ea4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5B55AC-A0C1-45C3-9411-3D2F7156D1B8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB7D7E8-8145-4A74-B49E-03C8140943AB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ceff588c-4f4f-49af-b7d7-c9c79415ad32"/>
+    <ds:schemaRef ds:uri="0ea24c86-fc74-4fa0-a83b-660477924ea4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB7D7E8-8145-4A74-B49E-03C8140943AB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5B55AC-A0C1-45C3-9411-3D2F7156D1B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Ruido/externo Longa duracao: montagem com fast (F) + 4 checks extras
So na NBR 10151 Longa duracao (externo comum nao muda):
- config do equipamento passa a incluir "fast (F)".
- Montagem ganha 4 checks: fonte de energia (bateria/rede); cabo de extensao
  validado (quando aplicavel); programar verificacoes intermediarias ao longo
  da campanha (quando aplicavel); verificar comunicacao com internet (online).

checksMontagemExterno(longaDuracao) (render + validacao). Cache ecamp-v0.7.9.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="120" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A839BED7-ADD2-4BFE-A667-046CD60D8FA6}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="8_{168677DE-32DB-4EA7-AD63-4473747FF806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C77CC868-61AE-48F6-8093-EF5F7321E6FF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="38">
   <si>
     <t>Ruído Ambiental – NBR 10151</t>
   </si>
@@ -170,9 +170,6 @@
   </si>
   <si>
     <t>Mantenha sempre as alterações e versões que ajustei nas conversas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documento de referência: </t>
   </si>
   <si>
     <t>e-CAMP</t>
@@ -286,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -300,34 +297,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -664,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9526D981-1FA4-46DC-815A-C9E12F5EFA92}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.21875" customWidth="1"/>
@@ -686,7 +687,7 @@
       <c r="C1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -696,177 +697,177 @@
         <v>29</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="14"/>
+      <c r="G2" s="15" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+    <row r="3" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="D3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="F3" s="14"/>
+      <c r="G3" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B4" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E4" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="14"/>
-      <c r="G3" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="14"/>
+      <c r="G4" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="D5" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="14"/>
-      <c r="G4" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="2" t="s">
+      <c r="F5" s="14"/>
+      <c r="G5" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="D6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="14"/>
-      <c r="G5" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="F6" s="14"/>
+      <c r="G6" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="B7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D7" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="F7" s="14"/>
+      <c r="G7" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="D8" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="F8" s="14"/>
+      <c r="G8" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D9" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E9" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>33</v>
-      </c>
       <c r="F9" s="14"/>
-      <c r="G9" s="7" t="s">
-        <v>38</v>
+      <c r="G9" s="15" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -875,7 +876,7 @@
       <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="7" t="s">
         <v>30</v>
       </c>
       <c r="E10" s="4" t="s">
@@ -884,10 +885,10 @@
       <c r="F10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="7"/>
+      <c r="G10" s="5"/>
     </row>
     <row r="11" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -896,7 +897,7 @@
       <c r="C11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="8" t="s">
         <v>30</v>
       </c>
       <c r="E11" s="4" t="s">
@@ -905,10 +906,10 @@
       <c r="F11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="7"/>
+      <c r="G11" s="5"/>
     </row>
     <row r="12" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -917,7 +918,7 @@
       <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="8" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="4" t="s">
@@ -926,10 +927,10 @@
       <c r="F12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="7"/>
+      <c r="G12" s="5"/>
     </row>
     <row r="13" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -938,7 +939,7 @@
       <c r="C13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="8" t="s">
         <v>30</v>
       </c>
       <c r="E13" s="4" t="s">
@@ -947,10 +948,10 @@
       <c r="F13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="7"/>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B14" s="2" t="s">
@@ -959,7 +960,7 @@
       <c r="C14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="8" t="s">
         <v>30</v>
       </c>
       <c r="E14" s="4" t="s">
@@ -968,10 +969,10 @@
       <c r="F14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="7"/>
+      <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -980,7 +981,7 @@
       <c r="C15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="8" t="s">
         <v>30</v>
       </c>
       <c r="E15" s="4" t="s">
@@ -989,84 +990,76 @@
       <c r="F15" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="7"/>
+      <c r="G15" s="5"/>
     </row>
     <row r="16" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
+      <c r="A16" s="8"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
     </row>
     <row r="17" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
+      <c r="A17" s="8"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
     </row>
     <row r="18" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
     </row>
     <row r="19" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
     </row>
     <row r="20" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
     </row>
     <row r="21" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
     </row>
     <row r="22" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
     </row>
     <row r="23" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>34</v>
+      </c>
       <c r="B23" t="s">
-        <v>34</v>
-      </c>
-      <c r="C23" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Outro (generico): tipo novo no eCamp
Conforme ecamp_especificacao.docx (romaneio 7.6, tela 8.6). Sem subtipo.
Geral: tipo de monitoramento (texto), objetivo, qtde de pontos. Por ponto:
nome, GPS, hora inicial, medicao principal + unidade, foto da tela + foto do
ponto, condicoes ambientais (temp/umid/vento com alerta >=5 m/s), observacoes.

- campo-outro.js (novo). romaneios.js: romaneio 'outro' (online opcional).
- fluxo.js: despacho, validacao, avisos e resumo da revisao.
- Equipamentos do tipo Outro seguem como cadastro manual (sem lista no F021).
- index.html + service-worker (cache v0.13.0).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engearlaboratorio.sharepoint.com/sites/EngearFinanceiro/Documentos Compartilhados/FINANCEIRO LAB/0 SISTEMA SGE/E-CAMP/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{83E09168-405E-41CC-B314-BC678F77B6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1CF8B34-AABF-4C96-A23E-F2943FBFC230}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{83E09168-405E-41CC-B314-BC678F77B6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2289503-A14A-45BF-9721-E330F0207856}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CD6052-B43C-4BA8-A7B7-6CEBB0E5B4CD}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="70">
   <si>
     <t>Ruído Ambiental – NBR 10151</t>
   </si>
@@ -295,7 +295,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -311,6 +311,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -390,7 +396,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -429,9 +435,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1316,38 +1323,37 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="18" t="s">
+      <c r="B28" s="11"/>
+      <c r="C28" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="3"/>
+      <c r="D28" s="11"/>
       <c r="E28" s="9" t="s">
         <v>64</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="G28" s="3"/>
+      <c r="G28" s="11" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="29" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="16"/>
-      <c r="E29" s="9" t="s">
+      <c r="E29" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="F29" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="G29" s="16"/>
     </row>
     <row r="30" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -1583,15 +1589,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ceff588c-4f4f-49af-b7d7-c9c79415ad32">
@@ -1600,6 +1597,15 @@
     <TaxCatchAll xmlns="0ea24c86-fc74-4fa0-a83b-660477924ea4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1622,14 +1628,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5B55AC-A0C1-45C3-9411-3D2F7156D1B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB7D7E8-8145-4A74-B49E-03C8140943AB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1638,4 +1636,12 @@
     <ds:schemaRef ds:uri="0ea24c86-fc74-4fa0-a83b-660477924ea4"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5B55AC-A0C1-45C3-9411-3D2F7156D1B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Tela inicial: OS reais do SGP (Buscar + Em andamento + Recentes)
Puxa as 33 OS reais do SGP (menu Propostas/Ordem de Servico) via nova rota
GET /api/monitoramento/os, com cache local (offline). Tela de escolha da OS
agora tem: busca por numero/cliente, secao 'Em andamento' (OS com servico ja
iniciado no servidor, compartilhada entre aparelhos) e 'Recentes' (ultimas 10
deste aparelho). Fallback para os exemplos quando ainda nao ha nada baixado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/escopo_metodo_os.xlsx
+++ b/planilhas/escopo_metodo_os.xlsx
@@ -1589,6 +1589,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ceff588c-4f4f-49af-b7d7-c9c79415ad32">
@@ -1597,15 +1606,6 @@
     <TaxCatchAll xmlns="0ea24c86-fc74-4fa0-a83b-660477924ea4" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1628,6 +1628,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5B55AC-A0C1-45C3-9411-3D2F7156D1B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB7D7E8-8145-4A74-B49E-03C8140943AB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1636,12 +1644,4 @@
     <ds:schemaRef ds:uri="0ea24c86-fc74-4fa0-a83b-660477924ea4"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D5B55AC-A0C1-45C3-9411-3D2F7156D1B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>